<commit_message>
Prepare v1.2.0 Tier-B evidence release candidate
</commit_message>
<xml_diff>
--- a/supplementary/Supplementary_Data_FINAL.xlsx
+++ b/supplementary/Supplementary_Data_FINAL.xlsx
@@ -2,16 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1_Grid_robustness" sheetId="1" r:id="R0f7b555d3ab54c10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S2_Heldout_states" sheetId="2" r:id="R026220579951476f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S3_Configuration_results" sheetId="3" r:id="R50c3cd24f41945c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S4_Decision_reuse_queries" sheetId="4" r:id="R22b87d88a2f947b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S5_Knowledge_conditions" sheetId="5" r:id="R8ea344f203fc46e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S6_Performance_measurements" sheetId="6" r:id="R66ef0defc72c4a1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S7_External_observations" sheetId="7" r:id="Re6182dfb51004f31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S8_E1_decision_audit" sheetId="8" r:id="Racdd54d0e1134895"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S9_E2_robustness" sheetId="9" r:id="Rbdfe2eb37d1f4137"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S10_E3_scalability" sheetId="10" r:id="Rb3325603c1a24f85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1_Grid_robustness" sheetId="1" r:id="Re76b8e53f88547e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S2_Heldout_states" sheetId="2" r:id="R2116b6c87f5144d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S3_Configuration_results" sheetId="3" r:id="R948493cc8a7b48f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S4_Decision_reuse_queries" sheetId="4" r:id="R96ce99b3e9fe446a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S5_Knowledge_conditions" sheetId="5" r:id="Rdea50dfe3da14e8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S6_Performance_measurements" sheetId="6" r:id="R01ca97c05f0a4e7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S7_External_observations" sheetId="7" r:id="R1eb23792fb6049c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S8_E1_decision_audit" sheetId="8" r:id="Rc6a7f75c8747488a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S9_E2_robustness" sheetId="9" r:id="Raaab7335c1794078"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S10_E3_scalability" sheetId="10" r:id="Rb131b8b369824581"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S11_B1_online_reopt" sheetId="11" r:id="R0ebce33729ae400b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S12_B2_near_boundary" sheetId="12" r:id="Refbd40a0bc844412"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S13_B3_terminal_tolerance" sheetId="13" r:id="R0f2acf2ea1dd4448"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -90,7 +93,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="56">
+  <x:cellXfs count="57">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -257,6 +260,9 @@
     <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1257,6 +1263,554 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="36" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="54" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="12" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B1" s="12" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="C1" s="12" t="str">
+        <x:v>Interpretation / scope</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="12" t="str">
+        <x:v>Recoverable starting states audited</x:v>
+      </x:c>
+      <x:c r="B2" s="12" t="n">
+        <x:v>407</x:v>
+      </x:c>
+      <x:c r="C2" s="12" t="str">
+        <x:v>Complete finite population; primary 3-pass/100-µm represented domain</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="12" t="str">
+        <x:v>Exact first-action agreement</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
+        <x:v>407/407</x:v>
+      </x:c>
+      <x:c r="C3" s="12" t="str">
+        <x:v>RPRA vs on-demand continuous remaining-horizon re-optimization</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="12" t="str">
+        <x:v>RPRA full-horizon completions</x:v>
+      </x:c>
+      <x:c r="B4" s="12" t="str">
+        <x:v>407/407</x:v>
+      </x:c>
+      <x:c r="C4" s="12" t="str">
+        <x:v>Frozen preserving-action policy</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="12" t="str">
+        <x:v>ONLINE-REOPT full-horizon completions</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="str">
+        <x:v>407/407</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="str">
+        <x:v>Same current-action grid, local physics, objective, and tie rule</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="12" t="str">
+        <x:v>Full three-pass sequence agreement</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="str">
+        <x:v>407/407</x:v>
+      </x:c>
+      <x:c r="C6" s="12" t="str">
+        <x:v>Exact action-sequence agreement for every start</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="12" t="str">
+        <x:v>RPRA-selected continuous-infeasible actions</x:v>
+      </x:c>
+      <x:c r="B7" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C7" s="12" t="str">
+        <x:v>No scientific-conflict case observed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="12" t="str">
+        <x:v>ONLINE-selected discrete-rejected actions</x:v>
+      </x:c>
+      <x:c r="B8" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C8" s="12" t="str">
+        <x:v>No selected online action fell outside the RPRA preserving envelope</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="12" t="str">
+        <x:v>Numerical unresolved outcomes</x:v>
+      </x:c>
+      <x:c r="B9" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C9" s="12" t="str">
+        <x:v>All scientific classifications resolved under the frozen validity rule</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="12" t="str">
+        <x:v>ONLINE downstream solves for 407 first decisions</x:v>
+      </x:c>
+      <x:c r="B10" s="12" t="n">
+        <x:v>42312</x:v>
+      </x:c>
+      <x:c r="C10" s="12" t="str">
+        <x:v>Structural uncached solve burden under the predeclared candidate-search rule</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="12" t="str">
+        <x:v>ONLINE solve calls per first decision, median</x:v>
+      </x:c>
+      <x:c r="B11" s="12" t="n">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="C11" s="12" t="str">
+        <x:v>Mean 103.961; P95 269.7; range 1-290</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="12" t="str">
+        <x:v>RPRA first-decision latency, pooled median (ms)</x:v>
+      </x:c>
+      <x:c r="B12" s="12" t="n">
+        <x:v>0.1717</x:v>
+      </x:c>
+      <x:c r="C12" s="12" t="str">
+        <x:v>41-state fixed subset; 1 warm-up + 5 measured runs/state</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="12" t="str">
+        <x:v>ONLINE-REOPT first-decision latency, pooled median (ms)</x:v>
+      </x:c>
+      <x:c r="B13" s="12" t="n">
+        <x:v>7080.9788</x:v>
+      </x:c>
+      <x:c r="C13" s="12" t="str">
+        <x:v>Same fixed subset and environment; uncached online evaluation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="12" t="str">
+        <x:v>Environment matches frozen E3</x:v>
+      </x:c>
+      <x:c r="B14" s="12" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="C14" s="12" t="str">
+        <x:v>Python 3.11.9; NumPy 2.4.6; SciPy 1.17.1; same OS/CPU/core counts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="12" t="str">
+        <x:v>Residual-valid SciPy non-success diagnostics</x:v>
+      </x:c>
+      <x:c r="B15" s="12" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="C15" s="12" t="str">
+        <x:v>26 classified PASS, 5 FAIL; all satisfy frozen residual-validity checks</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="12" t="str">
+        <x:v>B1 scientific classification</x:v>
+      </x:c>
+      <x:c r="B16" s="12" t="str">
+        <x:v>B1_STRONG_SUPPORT</x:v>
+      </x:c>
+      <x:c r="C16" s="12" t="str">
+        <x:v>Decision-equivalence evidence only; not optimizer superiority or universal equivalence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="12" t="str">
+        <x:v>Public-release note</x:v>
+      </x:c>
+      <x:c r="B17" s="12" t="str">
+        <x:v>v1.2.0 release candidate</x:v>
+      </x:c>
+      <x:c r="C17" s="12" t="str">
+        <x:v>Raw B1 audit files remain authoritative; public v1.1.0 is not modified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>Immediate-deflection sacrifice max (µm)</x:v>
+      </x:c>
+      <x:c r="B18" t="n">
+        <x:v>60.6540763821</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>All starts</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="21" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="40" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="12" t="str">
+        <x:v>Grid (mm)</x:v>
+      </x:c>
+      <x:c r="B1" s="12" t="str">
+        <x:v>Agreement</x:v>
+      </x:c>
+      <x:c r="C1" s="12" t="str">
+        <x:v>False rejection</x:v>
+      </x:c>
+      <x:c r="D1" s="56" t="str">
+        <x:v>False acceptance</x:v>
+      </x:c>
+      <x:c r="E1" s="56" t="str">
+        <x:v>Max error distance (µm)</x:v>
+      </x:c>
+      <x:c r="F1" s="56" t="str">
+        <x:v>Boundary under-approx. (µm)</x:v>
+      </x:c>
+      <x:c r="G1" s="56" t="str">
+        <x:v>Scope</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="12" t="n">
+        <x:v>0.004</x:v>
+      </x:c>
+      <x:c r="B2" s="12" t="str">
+        <x:v>112/161</x:v>
+      </x:c>
+      <x:c r="C2" s="12" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="D2" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E2" s="12" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F2" s="12" t="n">
+        <x:v>12.030453</x:v>
+      </x:c>
+      <x:c r="G2" s="12" t="str">
+        <x:v>161 states within ±20 µm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="12" t="n">
+        <x:v>0.002</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
+        <x:v>144/161</x:v>
+      </x:c>
+      <x:c r="C3" s="12" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D3" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E3" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F3" s="12" t="n">
+        <x:v>4.030453</x:v>
+      </x:c>
+      <x:c r="G3" s="12" t="str">
+        <x:v>161 states within ±20 µm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="12" t="n">
+        <x:v>0.001</x:v>
+      </x:c>
+      <x:c r="B4" s="12" t="str">
+        <x:v>152/161</x:v>
+      </x:c>
+      <x:c r="C4" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D4" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E4" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F4" s="12" t="n">
+        <x:v>2.030453</x:v>
+      </x:c>
+      <x:c r="G4" s="12" t="str">
+        <x:v>Adopted manuscript grid</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="12" t="n">
+        <x:v>0.0005</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="str">
+        <x:v>154/161</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E5" s="12" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="F5" s="12" t="n">
+        <x:v>1.530453</x:v>
+      </x:c>
+      <x:c r="G5" s="12" t="str">
+        <x:v>161 states within ±20 µm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="12" t="n">
+        <x:v>0.00025</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="str">
+        <x:v>158/161</x:v>
+      </x:c>
+      <x:c r="C6" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D6" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="12" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F6" s="12" t="n">
+        <x:v>0.530453</x:v>
+      </x:c>
+      <x:c r="G6" s="12" t="str">
+        <x:v>161 states within ±20 µm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="12" t="str">
+        <x:v>Classification</x:v>
+      </x:c>
+      <x:c r="B7" s="12" t="str">
+        <x:v>B2_STRONG_SUPPORT</x:v>
+      </x:c>
+      <x:c r="C7" s="12"/>
+      <x:c r="D7" s="12"/>
+      <x:c r="E7" s="12"/>
+      <x:c r="F7" s="12"/>
+      <x:c r="G7" s="12" t="str">
+        <x:v>Zero optimistic false acceptances and zero unresolved cases at all five grids</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="12" t="str">
+        <x:v>Case</x:v>
+      </x:c>
+      <x:c r="B1" s="12" t="str">
+        <x:v>Local feasible</x:v>
+      </x:c>
+      <x:c r="C1" s="12" t="str">
+        <x:v>Recoverable</x:v>
+      </x:c>
+      <x:c r="D1" s="56" t="str">
+        <x:v>Local but irrecoverable</x:v>
+      </x:c>
+      <x:c r="E1" s="56" t="str">
+        <x:v>Mixed-action</x:v>
+      </x:c>
+      <x:c r="F1" s="56" t="str">
+        <x:v>All-preserving</x:v>
+      </x:c>
+      <x:c r="G1" s="56" t="str">
+        <x:v>MYOPIC completion</x:v>
+      </x:c>
+      <x:c r="H1" s="56" t="str">
+        <x:v>RPRA completion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="12" t="str">
+        <x:v>T0 exact</x:v>
+      </x:c>
+      <x:c r="B2" s="12" t="n">
+        <x:v>621</x:v>
+      </x:c>
+      <x:c r="C2" s="12" t="n">
+        <x:v>407</x:v>
+      </x:c>
+      <x:c r="D2" s="12" t="n">
+        <x:v>214</x:v>
+      </x:c>
+      <x:c r="E2" s="12" t="n">
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="F2" s="12" t="n">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="G2" s="12" t="str">
+        <x:v>3/407</x:v>
+      </x:c>
+      <x:c r="H2" s="12" t="str">
+        <x:v>407/407</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="12" t="str">
+        <x:v>T5 ±5 µm</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="n">
+        <x:v>621</x:v>
+      </x:c>
+      <x:c r="C3" s="12" t="n">
+        <x:v>419</x:v>
+      </x:c>
+      <x:c r="D3" s="12" t="n">
+        <x:v>202</x:v>
+      </x:c>
+      <x:c r="E3" s="12" t="n">
+        <x:v>293</x:v>
+      </x:c>
+      <x:c r="F3" s="12" t="n">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="G3" s="12" t="str">
+        <x:v>9/419</x:v>
+      </x:c>
+      <x:c r="H3" s="12" t="str">
+        <x:v>419/419</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="12" t="str">
+        <x:v>T10 ±10 µm</x:v>
+      </x:c>
+      <x:c r="B4" s="12" t="n">
+        <x:v>621</x:v>
+      </x:c>
+      <x:c r="C4" s="12" t="n">
+        <x:v>431</x:v>
+      </x:c>
+      <x:c r="D4" s="12" t="n">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="E4" s="12" t="n">
+        <x:v>431</x:v>
+      </x:c>
+      <x:c r="F4" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G4" s="12" t="str">
+        <x:v>16/431</x:v>
+      </x:c>
+      <x:c r="H4" s="12" t="str">
+        <x:v>431/431</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="12" t="str">
+        <x:v>T20 ±20 µm</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="n">
+        <x:v>621</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="n">
+        <x:v>457</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="n">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="E5" s="12" t="n">
+        <x:v>457</x:v>
+      </x:c>
+      <x:c r="F5" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G5" s="12" t="str">
+        <x:v>29/457</x:v>
+      </x:c>
+      <x:c r="H5" s="12" t="str">
+        <x:v>457/457</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="12" t="str">
+        <x:v>Classification</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="str">
+        <x:v>B3_STRONG_SUPPORT</x:v>
+      </x:c>
+      <x:c r="C6" s="12"/>
+      <x:c r="D6" s="12"/>
+      <x:c r="E6" s="12"/>
+      <x:c r="F6" s="12"/>
+      <x:c r="G6" s="12"/>
+      <x:c r="H6" s="12" t="str">
+        <x:v>Separation persists across all declared terminal bands</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>

</xml_diff>